<commit_message>
Seed and synthetic data: invented names instead of real retail chains
The synthetic customer master (synth-data customers CSVs) named real
retail chains, and one word of the demo seed's grocery name pool was a
real chain's name. They are replaced by invented names. The two committed
order fixtures that used the pool word are regenerated with
pnpm fixtures:dispatch -- --date=2026-09-25: only those name cells change
(17 rows of orders-large.csv, 5 cells of orders-150.xlsx); the other
fixtures come out byte-identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/tests/fixtures/nmwc/orders-150.xlsx
+++ b/apps/web/tests/fixtures/nmwc/orders-150.xlsx
@@ -2249,7 +2249,7 @@
         <v/>
       </c>
       <c r="F53" t="str">
-        <v>Al Safa Grocery</v>
+        <v>Al Masa Grocery</v>
       </c>
       <c r="G53" t="str">
         <v>TAN-500-24</v>
@@ -2284,7 +2284,7 @@
         <v/>
       </c>
       <c r="F54" t="str">
-        <v>Al Safa Grocery</v>
+        <v>Al Masa Grocery</v>
       </c>
       <c r="G54" t="str">
         <v>TAN-1500-6</v>
@@ -2319,7 +2319,7 @@
         <v/>
       </c>
       <c r="F55" t="str">
-        <v>Al Safa Grocery</v>
+        <v>Al Masa Grocery</v>
       </c>
       <c r="G55" t="str">
         <v>TAN-330-24</v>
@@ -6764,7 +6764,7 @@
         <v/>
       </c>
       <c r="F182" t="str">
-        <v>Al Safa Foodstuff</v>
+        <v>Al Masa Foodstuff</v>
       </c>
       <c r="G182" t="str">
         <v>TAN-19L</v>
@@ -6799,7 +6799,7 @@
         <v/>
       </c>
       <c r="F183" t="str">
-        <v>Al Safa Foodstuff</v>
+        <v>Al Masa Foodstuff</v>
       </c>
       <c r="G183" t="str">
         <v>TIS-FAC-30</v>

</xml_diff>

<commit_message>
Tests and seed data: invented names for the last brand-like words
Review follow-up. A few invented shop names in the seed data, the
synthetic customer master and five test files still used one common
word that is also the brand word of a real customer chain, and one test
driver had a surname that is also a real chain's name. They now use
invented words; the Arabic test strings keep the same letter count and
the same Windows-1256 byte classes, so the decoding tests read the same.

The two committed order fixtures are regenerated with
pnpm fixtures:dispatch -- --date=2026-09-25: only 4 name cells change in
each of orders-large.csv and orders-150.xlsx; orders-20.csv and
late-p1.csv come out byte-identical. A solver test comment is reworded.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/tests/fixtures/nmwc/orders-150.xlsx
+++ b/apps/web/tests/fixtures/nmwc/orders-150.xlsx
@@ -7569,7 +7569,7 @@
         <v>B01</v>
       </c>
       <c r="F205" t="str">
-        <v>Al Noor Grocery - Ruwi</v>
+        <v>Al Nimr Grocery - Ruwi</v>
       </c>
       <c r="G205" t="str">
         <v>TAN-5L-4</v>
@@ -7604,7 +7604,7 @@
         <v>B01</v>
       </c>
       <c r="F206" t="str">
-        <v>Al Noor Grocery - Ruwi</v>
+        <v>Al Nimr Grocery - Ruwi</v>
       </c>
       <c r="G206" t="str">
         <v>TAN-500-24</v>
@@ -11909,7 +11909,7 @@
         <v>B02</v>
       </c>
       <c r="F329" t="str">
-        <v>Al Noor Grocery - Al Ansab</v>
+        <v>Al Nimr Grocery - Al Ansab</v>
       </c>
       <c r="G329" t="str">
         <v>TAN-1500-6</v>
@@ -11944,7 +11944,7 @@
         <v>B02</v>
       </c>
       <c r="F330" t="str">
-        <v>Al Noor Grocery - Al Ansab</v>
+        <v>Al Nimr Grocery - Al Ansab</v>
       </c>
       <c r="G330" t="str">
         <v>JAB-500-24</v>

</xml_diff>